<commit_message>
Shipping rates 1 pound update and support email address fix
</commit_message>
<xml_diff>
--- a/frontend/Revised Rates Newest.xlsx
+++ b/frontend/Revised Rates Newest.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\davja\OneDrive\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grush\Master\Package-Boss\frontend\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F24B36A7-5915-4E26-9FAB-9CC6DA79659F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="10512"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -52,11 +53,11 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="8" formatCode="&quot;$&quot;#,##0.00;[Red]\-&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00;[Red]\-&quot;$&quot;#,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -125,12 +126,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="8" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="8" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="8" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -464,15 +465,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H51"/>
-  <sheetFormatPr defaultRowHeight="13.8"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="14" customWidth="1"/>
     <col min="3" max="3" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -483,24 +484,24 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.6">
+    <row r="2" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="3">
-        <v>650</v>
+        <v>700</v>
       </c>
       <c r="C2" s="3">
         <f>B2/160</f>
-        <v>4.0625</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.6">
+        <v>4.375</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="3">
-        <f>B2+450</f>
+        <f>B2+400</f>
         <v>1100</v>
       </c>
       <c r="C3" s="3">
@@ -508,7 +509,7 @@
         <v>6.875</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.6">
+    <row r="4" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -521,7 +522,7 @@
         <v>9.375</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.6">
+    <row r="5" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -534,7 +535,7 @@
         <v>11.875</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.6">
+    <row r="6" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -547,7 +548,7 @@
         <v>14.6875</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.6">
+    <row r="7" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -560,7 +561,7 @@
         <v>17.1875</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.6">
+    <row r="8" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -573,7 +574,7 @@
         <v>19.6875</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.6">
+    <row r="9" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -586,7 +587,7 @@
         <v>22.1875</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.6">
+    <row r="10" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -599,7 +600,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.6">
+    <row r="11" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -612,7 +613,7 @@
         <v>29.0625</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.6">
+    <row r="12" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -625,7 +626,7 @@
         <v>31.5625</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.6">
+    <row r="13" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -638,7 +639,7 @@
         <v>34.375</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.6">
+    <row r="14" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -651,7 +652,7 @@
         <v>36.875</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.6">
+    <row r="15" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -664,7 +665,7 @@
         <v>39.375</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.6">
+    <row r="16" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -677,7 +678,7 @@
         <v>41.875</v>
       </c>
     </row>
-    <row r="17" spans="1:8" ht="15.6">
+    <row r="17" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -690,7 +691,7 @@
         <v>44.375</v>
       </c>
     </row>
-    <row r="18" spans="1:8" ht="15.6">
+    <row r="18" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -703,7 +704,7 @@
         <v>46.875</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="15.6">
+    <row r="19" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -716,7 +717,7 @@
         <v>49.6875</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="15.6">
+    <row r="20" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A20" s="2">
         <v>19</v>
       </c>
@@ -729,7 +730,7 @@
         <v>52.1875</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="15.6">
+    <row r="21" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -745,7 +746,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:8" ht="15.6">
+    <row r="22" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A22" s="2">
         <f>A21+1</f>
         <v>21</v>
@@ -759,7 +760,7 @@
         <v>57.1875</v>
       </c>
     </row>
-    <row r="23" spans="1:8" ht="15.6">
+    <row r="23" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A23" s="2">
         <f t="shared" ref="A23:A51" si="1">A22+1</f>
         <v>22</v>
@@ -773,7 +774,7 @@
         <v>60.3125</v>
       </c>
     </row>
-    <row r="24" spans="1:8" ht="15.6">
+    <row r="24" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A24" s="2">
         <f t="shared" si="1"/>
         <v>23</v>
@@ -787,7 +788,7 @@
         <v>62.1875</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="15.6">
+    <row r="25" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A25" s="2">
         <f t="shared" si="1"/>
         <v>24</v>
@@ -801,7 +802,7 @@
         <v>64.6875</v>
       </c>
     </row>
-    <row r="26" spans="1:8" ht="15.6">
+    <row r="26" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A26" s="2">
         <f t="shared" si="1"/>
         <v>25</v>
@@ -815,7 +816,7 @@
         <v>67.1875</v>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="15.6">
+    <row r="27" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A27" s="2">
         <f t="shared" si="1"/>
         <v>26</v>
@@ -829,7 +830,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="28" spans="1:8" ht="15.6">
+    <row r="28" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A28" s="2">
         <f t="shared" si="1"/>
         <v>27</v>
@@ -843,7 +844,7 @@
         <v>72.5</v>
       </c>
     </row>
-    <row r="29" spans="1:8" ht="15.6">
+    <row r="29" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A29" s="2">
         <f t="shared" si="1"/>
         <v>28</v>
@@ -857,7 +858,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="30" spans="1:8" ht="15.6">
+    <row r="30" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A30" s="2">
         <f t="shared" si="1"/>
         <v>29</v>
@@ -871,7 +872,7 @@
         <v>77.5</v>
       </c>
     </row>
-    <row r="31" spans="1:8" ht="15.6">
+    <row r="31" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <f t="shared" si="1"/>
         <v>30</v>
@@ -885,7 +886,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="32" spans="1:8" ht="15.6">
+    <row r="32" spans="1:8" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A32" s="2">
         <f t="shared" si="1"/>
         <v>31</v>
@@ -899,7 +900,7 @@
         <v>92.1875</v>
       </c>
     </row>
-    <row r="33" spans="1:3" ht="15.6">
+    <row r="33" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A33" s="2">
         <f t="shared" si="1"/>
         <v>32</v>
@@ -913,7 +914,7 @@
         <v>94.6875</v>
       </c>
     </row>
-    <row r="34" spans="1:3" ht="15.6">
+    <row r="34" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A34" s="2">
         <f t="shared" si="1"/>
         <v>33</v>
@@ -927,7 +928,7 @@
         <v>99.0625</v>
       </c>
     </row>
-    <row r="35" spans="1:3" ht="15.6">
+    <row r="35" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A35" s="2">
         <f t="shared" si="1"/>
         <v>34</v>
@@ -941,7 +942,7 @@
         <v>100.9375</v>
       </c>
     </row>
-    <row r="36" spans="1:3" ht="15.6">
+    <row r="36" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A36" s="2">
         <f t="shared" si="1"/>
         <v>35</v>
@@ -955,7 +956,7 @@
         <v>104.6875</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15.6">
+    <row r="37" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A37" s="2">
         <f t="shared" si="1"/>
         <v>36</v>
@@ -969,7 +970,7 @@
         <v>107.8125</v>
       </c>
     </row>
-    <row r="38" spans="1:3" ht="15.6">
+    <row r="38" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A38" s="2">
         <f t="shared" si="1"/>
         <v>37</v>
@@ -983,7 +984,7 @@
         <v>110.9375</v>
       </c>
     </row>
-    <row r="39" spans="1:3" ht="15.6">
+    <row r="39" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A39" s="2">
         <f t="shared" si="1"/>
         <v>38</v>
@@ -997,7 +998,7 @@
         <v>114.0625</v>
       </c>
     </row>
-    <row r="40" spans="1:3" ht="15.6">
+    <row r="40" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A40" s="2">
         <f t="shared" si="1"/>
         <v>39</v>
@@ -1011,7 +1012,7 @@
         <v>117.1875</v>
       </c>
     </row>
-    <row r="41" spans="1:3" ht="15.6">
+    <row r="41" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A41" s="2">
         <f t="shared" si="1"/>
         <v>40</v>
@@ -1025,7 +1026,7 @@
         <v>119.6875</v>
       </c>
     </row>
-    <row r="42" spans="1:3" ht="15.6">
+    <row r="42" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A42" s="2">
         <f t="shared" si="1"/>
         <v>41</v>
@@ -1039,7 +1040,7 @@
         <v>122.8125</v>
       </c>
     </row>
-    <row r="43" spans="1:3" ht="15.6">
+    <row r="43" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A43" s="2">
         <f t="shared" si="1"/>
         <v>42</v>
@@ -1053,7 +1054,7 @@
         <v>125.625</v>
       </c>
     </row>
-    <row r="44" spans="1:3" ht="15.6">
+    <row r="44" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A44" s="2">
         <f t="shared" si="1"/>
         <v>43</v>
@@ -1067,7 +1068,7 @@
         <v>128.4375</v>
       </c>
     </row>
-    <row r="45" spans="1:3" ht="15.6">
+    <row r="45" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A45" s="2">
         <f t="shared" si="1"/>
         <v>44</v>
@@ -1081,7 +1082,7 @@
         <v>131.875</v>
       </c>
     </row>
-    <row r="46" spans="1:3" ht="15.6">
+    <row r="46" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A46" s="2">
         <f t="shared" si="1"/>
         <v>45</v>
@@ -1095,7 +1096,7 @@
         <v>134.6875</v>
       </c>
     </row>
-    <row r="47" spans="1:3" ht="15.6">
+    <row r="47" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A47" s="2">
         <f t="shared" si="1"/>
         <v>46</v>
@@ -1109,7 +1110,7 @@
         <v>137.5</v>
       </c>
     </row>
-    <row r="48" spans="1:3" ht="15.6">
+    <row r="48" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A48" s="2">
         <f t="shared" si="1"/>
         <v>47</v>
@@ -1123,7 +1124,7 @@
         <v>140.625</v>
       </c>
     </row>
-    <row r="49" spans="1:3" ht="15.6">
+    <row r="49" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A49" s="2">
         <f t="shared" si="1"/>
         <v>48</v>
@@ -1137,7 +1138,7 @@
         <v>143.125</v>
       </c>
     </row>
-    <row r="50" spans="1:3" ht="15.6">
+    <row r="50" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A50" s="2">
         <f t="shared" si="1"/>
         <v>49</v>
@@ -1151,7 +1152,7 @@
         <v>146.875</v>
       </c>
     </row>
-    <row r="51" spans="1:3" ht="15.6">
+    <row r="51" spans="1:3" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A51" s="2">
         <f t="shared" si="1"/>
         <v>50</v>

</xml_diff>